<commit_message>
corrections and Textvergleich SSP
corrections of missing abbreviations
add missing IDs (addspan)
Textvergleich
add to Personenregister
</commit_message>
<xml_diff>
--- a/data/xlsx/Baernreither_Personenregister_2024.xlsx
+++ b/data/xlsx/Baernreither_Personenregister_2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christofaichner/Documents/GitHub/baernreither-data/data/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212C8CEE-292B-D249-8FC8-6D12DA7E6D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564A4656-AD60-7143-9AFC-618BCA59599C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5909" uniqueCount="4363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5910" uniqueCount="4363">
   <si>
     <t>Nachname</t>
   </si>
@@ -13003,9 +13003,6 @@
     <t>Scarpa</t>
   </si>
   <si>
-    <t>Generalagent des Öst. Lloyd in Bombay</t>
-  </si>
-  <si>
     <t>ScarpaEmil</t>
   </si>
   <si>
@@ -13283,6 +13280,9 @@
   </si>
   <si>
     <t>Hütten bei Königstein</t>
+  </si>
+  <si>
+    <t>Generalagent des Öst. Lloyd in Bombay, Rechtsanwalt und Verwaltungsrat</t>
   </si>
 </sst>
 </file>
@@ -14110,7 +14110,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="80" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="334">
+  <cellXfs count="335">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -14825,6 +14825,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -15925,13 +15928,13 @@
         <v>20</v>
       </c>
       <c r="H20" s="1" t="s">
+        <v>4328</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>4330</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>4329</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>4331</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>4330</v>
       </c>
     </row>
     <row r="21" spans="1:25" ht="32">
@@ -16773,7 +16776,7 @@
       </c>
       <c r="B41" s="1"/>
       <c r="C41" s="1" t="s">
-        <v>4351</v>
+        <v>4350</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1">
@@ -16781,14 +16784,14 @@
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1" t="s">
-        <v>4354</v>
+        <v>4353</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>4352</v>
+        <v>4351</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="1" t="s">
-        <v>4353</v>
+        <v>4352</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
@@ -22232,11 +22235,11 @@
       <c r="F176" s="25"/>
       <c r="G176" s="25"/>
       <c r="H176" s="26" t="s">
-        <v>4344</v>
+        <v>4343</v>
       </c>
       <c r="I176" s="184"/>
       <c r="J176" s="25" t="s">
-        <v>4345</v>
+        <v>4344</v>
       </c>
       <c r="K176" s="9"/>
       <c r="L176" s="9"/>
@@ -22267,11 +22270,11 @@
       <c r="F177" s="25"/>
       <c r="G177" s="25"/>
       <c r="H177" s="26" t="s">
-        <v>4346</v>
+        <v>4345</v>
       </c>
       <c r="I177" s="184"/>
       <c r="J177" s="25" t="s">
-        <v>4355</v>
+        <v>4354</v>
       </c>
       <c r="K177" s="9"/>
       <c r="L177" s="9"/>
@@ -22772,7 +22775,7 @@
     </row>
     <row r="191" spans="1:26" ht="15.75" customHeight="1">
       <c r="A191" s="2" t="s">
-        <v>4336</v>
+        <v>4335</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>731</v>
@@ -22793,13 +22796,13 @@
         <v>20</v>
       </c>
       <c r="H191" s="2" t="s">
+        <v>4336</v>
+      </c>
+      <c r="I191" s="180" t="s">
         <v>4337</v>
       </c>
-      <c r="I191" s="180" t="s">
+      <c r="J191" s="252" t="s">
         <v>4338</v>
-      </c>
-      <c r="J191" s="252" t="s">
-        <v>4339</v>
       </c>
       <c r="K191" s="1"/>
       <c r="L191" s="1"/>
@@ -26059,13 +26062,13 @@
     </row>
     <row r="277" spans="1:26" ht="15.75" customHeight="1">
       <c r="A277" s="1" t="s">
-        <v>4340</v>
+        <v>4339</v>
       </c>
       <c r="B277" s="1" t="s">
         <v>4222</v>
       </c>
       <c r="C277" s="1" t="s">
-        <v>4341</v>
+        <v>4340</v>
       </c>
       <c r="D277" s="1">
         <v>1886</v>
@@ -26080,11 +26083,11 @@
         <v>95</v>
       </c>
       <c r="H277" s="1" t="s">
-        <v>4342</v>
+        <v>4341</v>
       </c>
       <c r="I277" s="1"/>
       <c r="J277" s="75" t="s">
-        <v>4343</v>
+        <v>4342</v>
       </c>
       <c r="K277" s="75"/>
       <c r="L277" s="75"/>
@@ -27957,7 +27960,7 @@
     </row>
     <row r="322" spans="1:25" ht="15.75" customHeight="1">
       <c r="A322" s="15" t="s">
-        <v>4347</v>
+        <v>4346</v>
       </c>
       <c r="C322" s="15" t="s">
         <v>745</v>
@@ -27969,27 +27972,27 @@
         <v>1908</v>
       </c>
       <c r="F322" s="15" t="s">
-        <v>4362</v>
+        <v>4361</v>
       </c>
       <c r="G322" s="15" t="s">
         <v>419</v>
       </c>
       <c r="H322" s="15" t="s">
-        <v>4357</v>
+        <v>4356</v>
       </c>
       <c r="J322" s="15" t="s">
-        <v>4356</v>
+        <v>4355</v>
       </c>
     </row>
     <row r="323" spans="1:25" ht="15.75" customHeight="1">
       <c r="A323" s="15" t="s">
+        <v>4346</v>
+      </c>
+      <c r="B323" s="15" t="s">
+        <v>4360</v>
+      </c>
+      <c r="C323" t="s">
         <v>4347</v>
-      </c>
-      <c r="B323" s="15" t="s">
-        <v>4361</v>
-      </c>
-      <c r="C323" t="s">
-        <v>4348</v>
       </c>
       <c r="D323">
         <v>1857</v>
@@ -28004,15 +28007,15 @@
         <v>304</v>
       </c>
       <c r="H323" s="15" t="s">
+        <v>4348</v>
+      </c>
+      <c r="J323" s="15" t="s">
         <v>4349</v>
-      </c>
-      <c r="J323" s="15" t="s">
-        <v>4350</v>
       </c>
     </row>
     <row r="324" spans="1:25" ht="15.75" customHeight="1">
       <c r="A324" s="15" t="s">
-        <v>4347</v>
+        <v>4346</v>
       </c>
       <c r="C324" s="15" t="s">
         <v>143</v>
@@ -28030,13 +28033,13 @@
         <v>3672</v>
       </c>
       <c r="H324" s="15" t="s">
+        <v>4357</v>
+      </c>
+      <c r="I324" t="s">
+        <v>4359</v>
+      </c>
+      <c r="J324" s="15" t="s">
         <v>4358</v>
-      </c>
-      <c r="I324" t="s">
-        <v>4360</v>
-      </c>
-      <c r="J324" s="15" t="s">
-        <v>4359</v>
       </c>
     </row>
     <row r="325" spans="1:25" ht="15.75" customHeight="1">
@@ -30798,19 +30801,19 @@
         <v>1910</v>
       </c>
       <c r="F394" s="1" t="s">
-        <v>4332</v>
+        <v>4331</v>
       </c>
       <c r="G394" s="1" t="s">
         <v>20</v>
       </c>
       <c r="H394" s="1" t="s">
+        <v>4332</v>
+      </c>
+      <c r="I394" s="1" t="s">
         <v>4333</v>
       </c>
-      <c r="I394" s="1" t="s">
+      <c r="J394" s="1" t="s">
         <v>4334</v>
-      </c>
-      <c r="J394" s="1" t="s">
-        <v>4335</v>
       </c>
       <c r="K394" s="1"/>
       <c r="L394" s="1"/>
@@ -37953,11 +37956,11 @@
       <c r="F575" s="2"/>
       <c r="G575" s="2"/>
       <c r="H575" s="2" t="s">
-        <v>4327</v>
+        <v>4326</v>
       </c>
       <c r="I575" s="19"/>
       <c r="J575" s="2" t="s">
-        <v>4328</v>
+        <v>4327</v>
       </c>
       <c r="K575" s="10"/>
       <c r="L575" s="10"/>
@@ -40402,11 +40405,17 @@
       <c r="C639" t="s">
         <v>1038</v>
       </c>
-      <c r="H639" s="137" t="s">
+      <c r="E639">
+        <v>1929</v>
+      </c>
+      <c r="G639" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="H639" s="334" t="s">
+        <v>4362</v>
+      </c>
+      <c r="J639" t="s">
         <v>4269</v>
-      </c>
-      <c r="J639" t="s">
-        <v>4270</v>
       </c>
     </row>
     <row r="640" spans="1:25" ht="15.75" customHeight="1">
@@ -41072,7 +41081,7 @@
     </row>
     <row r="656" spans="1:25" ht="15.75" customHeight="1">
       <c r="A656" t="s">
-        <v>4271</v>
+        <v>4270</v>
       </c>
       <c r="C656" t="s">
         <v>151</v>
@@ -41084,19 +41093,19 @@
         <v>1927</v>
       </c>
       <c r="F656" t="s">
+        <v>4271</v>
+      </c>
+      <c r="G656" t="s">
         <v>4272</v>
       </c>
-      <c r="G656" t="s">
+      <c r="H656" s="137" t="s">
         <v>4273</v>
       </c>
-      <c r="H656" s="137" t="s">
+      <c r="I656" t="s">
         <v>4274</v>
       </c>
-      <c r="I656" t="s">
+      <c r="J656" t="s">
         <v>4275</v>
-      </c>
-      <c r="J656" t="s">
-        <v>4276</v>
       </c>
     </row>
     <row r="657" spans="1:25" ht="15.75" customHeight="1">
@@ -41712,7 +41721,7 @@
     </row>
     <row r="672" spans="1:25" ht="15.75" customHeight="1">
       <c r="A672" t="s">
-        <v>4277</v>
+        <v>4276</v>
       </c>
       <c r="C672" t="s">
         <v>432</v>
@@ -41730,13 +41739,13 @@
         <v>3621</v>
       </c>
       <c r="H672" s="137" t="s">
+        <v>4277</v>
+      </c>
+      <c r="I672" t="s">
         <v>4278</v>
       </c>
-      <c r="I672" t="s">
+      <c r="J672" t="s">
         <v>4279</v>
-      </c>
-      <c r="J672" t="s">
-        <v>4280</v>
       </c>
     </row>
     <row r="673" spans="1:25" ht="15.75" customHeight="1">
@@ -42872,7 +42881,7 @@
     </row>
     <row r="702" spans="1:25" ht="15.75" customHeight="1">
       <c r="A702" t="s">
-        <v>4281</v>
+        <v>4280</v>
       </c>
       <c r="C702" t="s">
         <v>1914</v>
@@ -42890,13 +42899,13 @@
         <v>1966</v>
       </c>
       <c r="H702" s="137" t="s">
+        <v>4281</v>
+      </c>
+      <c r="I702" s="124" t="s">
         <v>4282</v>
       </c>
-      <c r="I702" s="124" t="s">
+      <c r="J702" t="s">
         <v>4283</v>
-      </c>
-      <c r="J702" t="s">
-        <v>4284</v>
       </c>
     </row>
     <row r="703" spans="1:25" ht="15.75" customHeight="1">
@@ -44788,7 +44797,7 @@
     </row>
     <row r="751" spans="1:25" ht="15.75" customHeight="1">
       <c r="A751" t="s">
-        <v>4285</v>
+        <v>4284</v>
       </c>
       <c r="C751" t="s">
         <v>1050</v>
@@ -44806,13 +44815,13 @@
         <v>20</v>
       </c>
       <c r="H751" s="137" t="s">
+        <v>4285</v>
+      </c>
+      <c r="I751" t="s">
         <v>4286</v>
       </c>
-      <c r="I751" t="s">
+      <c r="J751" t="s">
         <v>4287</v>
-      </c>
-      <c r="J751" t="s">
-        <v>4288</v>
       </c>
     </row>
     <row r="752" spans="1:25" ht="15.75" customHeight="1">
@@ -45106,7 +45115,7 @@
     </row>
     <row r="759" spans="1:25" ht="15.75" customHeight="1">
       <c r="A759" t="s">
-        <v>4289</v>
+        <v>4288</v>
       </c>
       <c r="C759" t="s">
         <v>473</v>
@@ -45121,16 +45130,16 @@
         <v>1508</v>
       </c>
       <c r="G759" t="s">
+        <v>4289</v>
+      </c>
+      <c r="H759" s="137" t="s">
         <v>4290</v>
       </c>
-      <c r="H759" s="137" t="s">
+      <c r="I759" t="s">
         <v>4291</v>
       </c>
-      <c r="I759" t="s">
+      <c r="J759" t="s">
         <v>4292</v>
-      </c>
-      <c r="J759" t="s">
-        <v>4293</v>
       </c>
     </row>
     <row r="760" spans="1:25" ht="15.75" customHeight="1">
@@ -45290,10 +45299,10 @@
     </row>
     <row r="764" spans="1:25" ht="15.75" customHeight="1">
       <c r="A764" t="s">
+        <v>4293</v>
+      </c>
+      <c r="C764" t="s">
         <v>4294</v>
-      </c>
-      <c r="C764" t="s">
-        <v>4295</v>
       </c>
       <c r="D764">
         <v>1843</v>
@@ -45302,16 +45311,16 @@
         <v>1906</v>
       </c>
       <c r="F764" t="s">
-        <v>4296</v>
+        <v>4295</v>
       </c>
       <c r="G764" t="s">
         <v>1508</v>
       </c>
       <c r="H764" s="137" t="s">
+        <v>4296</v>
+      </c>
+      <c r="J764" t="s">
         <v>4297</v>
-      </c>
-      <c r="J764" t="s">
-        <v>4298</v>
       </c>
     </row>
     <row r="765" spans="1:25" ht="15.75" customHeight="1">
@@ -46207,10 +46216,10 @@
     </row>
     <row r="790" spans="1:25" ht="15.75" customHeight="1">
       <c r="A790" t="s">
+        <v>4298</v>
+      </c>
+      <c r="C790" t="s">
         <v>4299</v>
-      </c>
-      <c r="C790" t="s">
-        <v>4300</v>
       </c>
       <c r="D790">
         <v>1827</v>
@@ -46225,13 +46234,13 @@
         <v>800</v>
       </c>
       <c r="H790" s="137" t="s">
+        <v>4300</v>
+      </c>
+      <c r="I790" t="s">
         <v>4301</v>
       </c>
-      <c r="I790" t="s">
+      <c r="J790" t="s">
         <v>4302</v>
-      </c>
-      <c r="J790" t="s">
-        <v>4303</v>
       </c>
     </row>
     <row r="791" spans="1:25" ht="15.75" customHeight="1">
@@ -46283,13 +46292,13 @@
     </row>
     <row r="792" spans="1:25" ht="15.75" customHeight="1">
       <c r="A792" t="s">
+        <v>4303</v>
+      </c>
+      <c r="B792" t="s">
         <v>4304</v>
       </c>
-      <c r="B792" t="s">
+      <c r="C792" t="s">
         <v>4305</v>
-      </c>
-      <c r="C792" t="s">
-        <v>4306</v>
       </c>
       <c r="D792">
         <v>1877</v>
@@ -46298,19 +46307,19 @@
         <v>1953</v>
       </c>
       <c r="F792" t="s">
-        <v>4307</v>
+        <v>4306</v>
       </c>
       <c r="G792" t="s">
         <v>1204</v>
       </c>
       <c r="H792" s="137" t="s">
+        <v>4307</v>
+      </c>
+      <c r="I792" s="124" t="s">
         <v>4308</v>
       </c>
-      <c r="I792" s="124" t="s">
+      <c r="J792" t="s">
         <v>4309</v>
-      </c>
-      <c r="J792" t="s">
-        <v>4310</v>
       </c>
     </row>
     <row r="793" spans="1:25" ht="15.75" customHeight="1">
@@ -46391,7 +46400,7 @@
     </row>
     <row r="795" spans="1:25" ht="15.75" customHeight="1">
       <c r="A795" t="s">
-        <v>4311</v>
+        <v>4310</v>
       </c>
       <c r="B795" t="s">
         <v>26</v>
@@ -46406,19 +46415,19 @@
         <v>1930</v>
       </c>
       <c r="F795" t="s">
+        <v>4311</v>
+      </c>
+      <c r="G795" t="s">
         <v>4312</v>
       </c>
-      <c r="G795" t="s">
+      <c r="H795" s="137" t="s">
         <v>4313</v>
       </c>
-      <c r="H795" s="137" t="s">
+      <c r="I795" t="s">
         <v>4314</v>
       </c>
-      <c r="I795" t="s">
+      <c r="J795" t="s">
         <v>4315</v>
-      </c>
-      <c r="J795" t="s">
-        <v>4316</v>
       </c>
     </row>
     <row r="796" spans="1:25" ht="15.75" customHeight="1">
@@ -47496,13 +47505,13 @@
     </row>
     <row r="823" spans="1:25" ht="15.75" customHeight="1">
       <c r="A823" t="s">
-        <v>4317</v>
+        <v>4316</v>
       </c>
       <c r="B823" t="s">
         <v>18</v>
       </c>
       <c r="C823" t="s">
-        <v>4318</v>
+        <v>4317</v>
       </c>
       <c r="D823">
         <v>1838</v>
@@ -47517,13 +47526,13 @@
         <v>122</v>
       </c>
       <c r="H823" s="137" t="s">
+        <v>4318</v>
+      </c>
+      <c r="I823" t="s">
         <v>4319</v>
       </c>
-      <c r="I823" t="s">
+      <c r="J823" t="s">
         <v>4320</v>
-      </c>
-      <c r="J823" t="s">
-        <v>4321</v>
       </c>
     </row>
     <row r="824" spans="1:25" ht="15.75" customHeight="1">
@@ -47677,10 +47686,10 @@
     </row>
     <row r="828" spans="1:25" ht="15.75" customHeight="1">
       <c r="A828" t="s">
+        <v>4321</v>
+      </c>
+      <c r="C828" t="s">
         <v>4322</v>
-      </c>
-      <c r="C828" t="s">
-        <v>4323</v>
       </c>
       <c r="D828">
         <v>1819</v>
@@ -47695,13 +47704,13 @@
         <v>420</v>
       </c>
       <c r="H828" s="137" t="s">
+        <v>4323</v>
+      </c>
+      <c r="I828" t="s">
         <v>4324</v>
       </c>
-      <c r="I828" t="s">
+      <c r="J828" t="s">
         <v>4325</v>
-      </c>
-      <c r="J828" t="s">
-        <v>4326</v>
       </c>
     </row>
     <row r="829" spans="1:25" ht="15.75" customHeight="1">

</xml_diff>